<commit_message>
introduction sheet group order + reserve officials.
</commit_message>
<xml_diff>
--- a/owlcms/src/main/resources/templates/introduction/Introduction.xlsx
+++ b/owlcms/src/main/resources/templates/introduction/Introduction.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28623"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28730"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lamyj\git\owlcms4\owlcms\src\main\resources\templates\introduction\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D8D3828-4D4E-4CE2-9F5D-C6D3CF29E63E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3947B86E-9DCD-44A8-B99C-BBCB010B6435}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -64,51 +64,11 @@
             <rFont val="Aptos Narrow"/>
           </rPr>
           <t xml:space="preserve">jx:each(
-</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="12"/>
-            <color rgb="FF000000"/>
-            <rFont val="Aptos Narrow"/>
-          </rPr>
-          <t xml:space="preserve">  items="athletes"
-</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="12"/>
-            <color rgb="FF000000"/>
-            <rFont val="Aptos Narrow"/>
-          </rPr>
-          <t xml:space="preserve">  var="groups"
-</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="12"/>
-            <color rgb="FF000000"/>
-            <rFont val="Aptos Narrow"/>
-          </rPr>
-          <t xml:space="preserve">  groupBy="groups.longCategory"
-</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="12"/>
-            <color rgb="FF000000"/>
-            <rFont val="Aptos Narrow"/>
-          </rPr>
-          <t xml:space="preserve">  lastCell="J7"
-</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="12"/>
-            <color rgb="FF000000"/>
-            <rFont val="Aptos Narrow"/>
-          </rPr>
-          <t xml:space="preserve">)
+  items="athletes"
+  var="groups"
+  groupBy="groups.category.sortCode"
+  lastCell="J7"
+)
 </t>
         </r>
       </text>
@@ -171,7 +131,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="44">
   <si>
     <t>${competition.competitionName}</t>
   </si>
@@ -248,9 +208,6 @@
     <t>${t.get("CenterReferee")}</t>
   </si>
   <si>
-    <t>${t.get("Referee")}</t>
-  </si>
-  <si>
     <t>${session.announcerAsTO}</t>
   </si>
   <si>
@@ -291,6 +248,21 @@
   </si>
   <si>
     <t>${session.jury5AsTO}</t>
+  </si>
+  <si>
+    <t>${t.get("SideReferee")}</t>
+  </si>
+  <si>
+    <t>${t.get("ReserveReferee")}</t>
+  </si>
+  <si>
+    <t>${session.reserveAsTO}</t>
+  </si>
+  <si>
+    <t>${t.get("ReserveJury")}</t>
+  </si>
+  <si>
+    <t>${session.reserveJuryAsTO}</t>
   </si>
 </sst>
 </file>
@@ -947,68 +919,67 @@
         <v>24</v>
       </c>
       <c r="C10" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="F10" s="18" t="s">
         <v>19</v>
       </c>
       <c r="G10" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="11" spans="1:18" x14ac:dyDescent="0.25">
       <c r="B11" s="18" t="s">
-        <v>25</v>
+        <v>39</v>
       </c>
       <c r="C11" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F11" s="18" t="s">
         <v>21</v>
       </c>
       <c r="G11" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="12" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B12" s="18" t="s">
-        <v>25</v>
+        <v>39</v>
       </c>
       <c r="C12" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="F12" s="18" t="s">
         <v>21</v>
       </c>
       <c r="G12" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="O12" s="18"/>
       <c r="R12" s="23"/>
     </row>
     <row r="13" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B13" s="18"/>
+      <c r="B13" s="18" t="s">
+        <v>40</v>
+      </c>
+      <c r="C13" t="s">
+        <v>41</v>
+      </c>
       <c r="F13" s="18" t="s">
         <v>21</v>
       </c>
       <c r="G13" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="O13" s="18"/>
       <c r="R13" s="23"/>
     </row>
     <row r="14" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="B14" s="21" t="s">
-        <v>20</v>
-      </c>
-      <c r="C14" t="s">
-        <v>27</v>
-      </c>
       <c r="F14" s="18" t="s">
         <v>21</v>
       </c>
       <c r="G14" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="N14" s="18"/>
       <c r="O14" s="18"/>
@@ -1020,41 +991,47 @@
         <v>20</v>
       </c>
       <c r="C15" t="s">
-        <v>28</v>
+        <v>26</v>
+      </c>
+      <c r="F15" s="18" t="s">
+        <v>42</v>
+      </c>
+      <c r="G15" t="s">
+        <v>43</v>
       </c>
       <c r="K15" s="19"/>
       <c r="N15" s="22"/>
       <c r="O15" s="19"/>
     </row>
     <row r="16" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="B16" s="21"/>
-      <c r="F16" s="18" t="s">
-        <v>18</v>
-      </c>
-      <c r="G16" t="s">
-        <v>26</v>
+      <c r="B16" s="21" t="s">
+        <v>20</v>
+      </c>
+      <c r="C16" t="s">
+        <v>27</v>
       </c>
       <c r="K16" s="19"/>
       <c r="N16" s="22"/>
       <c r="O16" s="19"/>
     </row>
     <row r="17" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B17" s="18" t="s">
-        <v>22</v>
-      </c>
-      <c r="C17" t="s">
-        <v>29</v>
+      <c r="B17" s="21"/>
+      <c r="F17" s="18" t="s">
+        <v>18</v>
+      </c>
+      <c r="G17" t="s">
+        <v>25</v>
       </c>
       <c r="K17" s="20"/>
       <c r="N17" s="18"/>
       <c r="O17" s="18"/>
     </row>
     <row r="18" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B18" s="21" t="s">
-        <v>23</v>
+      <c r="B18" s="18" t="s">
+        <v>22</v>
       </c>
       <c r="C18" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="N18" s="18"/>
       <c r="O18" s="18"/>
@@ -1064,12 +1041,18 @@
         <v>23</v>
       </c>
       <c r="C19" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="N19" s="18"/>
       <c r="O19" s="18"/>
     </row>
     <row r="20" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B20" s="21" t="s">
+        <v>23</v>
+      </c>
+      <c r="C20" t="s">
+        <v>33</v>
+      </c>
       <c r="K20" s="19"/>
     </row>
     <row r="21" spans="2:15" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
update introduction sheet; closes #1312
</commit_message>
<xml_diff>
--- a/owlcms/src/main/resources/templates/introduction/Introduction.xlsx
+++ b/owlcms/src/main/resources/templates/introduction/Introduction.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29127"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lamyj\git\owlcms4\owlcms\src\main\resources\templates\introduction\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\git\owlcms_v23\owlcms\src\main\resources\templates\introduction\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8EFEB98A-41AF-4CD9-90B3-4A2465A9CAB1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B4FE1224-3484-48A9-9038-B33E1469ADC7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="5295" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -50,7 +50,7 @@
             <family val="2"/>
           </rPr>
           <t>jx:area(
-  lastCell="J28"
+  lastCell="J20"
 )</t>
         </r>
       </text>
@@ -131,14 +131,11 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="51">
   <si>
     <t>${competition.competitionName}</t>
   </si>
   <si>
-    <t>${session.localizedStartHour}</t>
-  </si>
-  <si>
     <t>${athlete.startNumber}</t>
   </si>
   <si>
@@ -160,9 +157,6 @@
     <t>${athlete.fullName}</t>
   </si>
   <si>
-    <t>${session.localizedStartDay}</t>
-  </si>
-  <si>
     <t>${t.get("Age")}</t>
   </si>
   <si>
@@ -172,9 +166,6 @@
     <t>${t.get("Clean_and_Jerk_short")}</t>
   </si>
   <si>
-    <t>${t.get("Group")} ${session.name} - ${session.ageGroupInfo.0.formattedRange}</t>
-  </si>
-  <si>
     <t>${tf.format("Break.MinutesBeforeCJ", session.cleanJerkBreakMinutes)}</t>
   </si>
   <si>
@@ -187,90 +178,119 @@
     <t>${groups.item.category}</t>
   </si>
   <si>
-    <t>${t.get("Announcer")}</t>
-  </si>
-  <si>
-    <t>${t.get("JuryPresident")}</t>
-  </si>
-  <si>
-    <t>${t.get("Marshall")}</t>
-  </si>
-  <si>
-    <t>${t.get("Jury")}</t>
-  </si>
-  <si>
-    <t>${t.get("Timekeeper")}</t>
-  </si>
-  <si>
-    <t>${t.get("Results.Controller")}</t>
-  </si>
-  <si>
-    <t>${t.get("CenterReferee")}</t>
-  </si>
-  <si>
-    <t>${session.announcerAsTO}</t>
-  </si>
-  <si>
-    <t xml:space="preserve">${session.marshallAsTO} </t>
-  </si>
-  <si>
-    <t>${session.marshal2AsTO}</t>
-  </si>
-  <si>
-    <t>${session.timeKeeperAsTO}</t>
-  </si>
-  <si>
-    <t>${session.referee2AsTO}</t>
-  </si>
-  <si>
-    <t>${session.referee1AsTO}</t>
-  </si>
-  <si>
-    <t>${session.referee3AsTO}</t>
-  </si>
-  <si>
-    <t>${session.technicalControllerAsTO}</t>
-  </si>
-  <si>
-    <t xml:space="preserve">${session.technicalController2AsTO} </t>
-  </si>
-  <si>
-    <t>${session.jury1AsTO}</t>
-  </si>
-  <si>
-    <t>${session.jury2AsTO}</t>
-  </si>
-  <si>
-    <t>${session.jury3AsTO}</t>
-  </si>
-  <si>
-    <t>${session.jury4AsTO}</t>
-  </si>
-  <si>
-    <t>${session.jury5AsTO}</t>
-  </si>
-  <si>
-    <t>${t.get("SideReferee")}</t>
-  </si>
-  <si>
-    <t>${t.get("ReserveReferee")}</t>
-  </si>
-  <si>
-    <t>${session.reserveAsTO}</t>
-  </si>
-  <si>
-    <t>${t.get("ReserveJury")}</t>
-  </si>
-  <si>
-    <t>${session.reserveJuryAsTO}</t>
+    <t>${session.referee2AsTO != null ? t.get("CenterReferee") : ""}</t>
+  </si>
+  <si>
+    <t>${session.referee1AsTO != null ? t.get("SideReferee"): ""}</t>
+  </si>
+  <si>
+    <t>${session.referee3AsTO != null ? t.get("SideReferee") : ""}</t>
+  </si>
+  <si>
+    <t>${session.reserveAsTO != null ? t.get("ReserveReferee") : ""}</t>
+  </si>
+  <si>
+    <t>${session.marshallAsTO != null ? t.get("Marshall") : ""}</t>
+  </si>
+  <si>
+    <t>${session.marshal2AsTO != null ? t.get("Marshall") : ""}</t>
+  </si>
+  <si>
+    <t>${session.timeKeeperAsTO != null ? t.get("Timekeeper") : ""}</t>
+  </si>
+  <si>
+    <t>${session.technicalControllerAsTO != null ? t.get("Results.Controller") : ""}</t>
+  </si>
+  <si>
+    <t>${session.technicalController2AsTO != null ? t.get("Results.Controller") : ""}</t>
+  </si>
+  <si>
+    <t>${session.jury1AsTO != null ? t.get("JuryPresident") : ""}</t>
+  </si>
+  <si>
+    <t>${session.reserveJuryAsTO != null ? t.get("ReserveJury") : ""}</t>
+  </si>
+  <si>
+    <t>${session.jury2AsTO != null ? t.get("Jury") : ""}</t>
+  </si>
+  <si>
+    <t>${session.jury3AsTO != null ? t.get("Jury") : ""}</t>
+  </si>
+  <si>
+    <t>${session.jury4AsTO != null ? t.get("Jury") : ""}</t>
+  </si>
+  <si>
+    <t>${session.jury5AsTO != null ? t.get("Jury") : ""}</t>
+  </si>
+  <si>
+    <t>${session.doctorAsTO != null ? t.get("Doctor") : ""}</t>
+  </si>
+  <si>
+    <t>${session.announcerAsTO != null ? t.get("Announcer") : ""}</t>
+  </si>
+  <si>
+    <t>${t.get("Group")} ${session.name} - ${session.ageGroupInfo.0.formattedRange} - ${session.description}</t>
+  </si>
+  <si>
+    <t>${session.localizedStartDay} ${session.localizedStartHour}</t>
+  </si>
+  <si>
+    <t>${session.referee2AsTO} ${session.referee2AsTO.federation}</t>
+  </si>
+  <si>
+    <t>${session.referee1AsTO} ${session.referee1AsTO.federation}</t>
+  </si>
+  <si>
+    <t>${session.referee3AsTO} ${session.referee3AsTO.federation}</t>
+  </si>
+  <si>
+    <t>${session.reserveAsTO} ${session.reserveAsT.federation}</t>
+  </si>
+  <si>
+    <t>${session.marshallAsTO} ${session.marshallAsTO.federation}</t>
+  </si>
+  <si>
+    <t>${session.marshal2AsTO} ${session.marshal2AsTO.federation}</t>
+  </si>
+  <si>
+    <t>${session.timeKeeperAsTO} ${session.timeKeeperAsTO.federation}</t>
+  </si>
+  <si>
+    <t>${session.technicalControllerAsTO} ${session.technicalControllerAsTO.federation}</t>
+  </si>
+  <si>
+    <t>${session.technicalController2AsTO} ${session.technicalController2AsTO.federation}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">${session.jury1AsTO} ${session.jury1AsTO.federation} </t>
+  </si>
+  <si>
+    <t>${session.jury2AsTO} ${session.jury2AsTO.federation}</t>
+  </si>
+  <si>
+    <t>${session.jury3AsTO} ${session.jury3AsTO.federation}</t>
+  </si>
+  <si>
+    <t>${session.jury4AsTO} ${session.jury4AsTO.federation}</t>
+  </si>
+  <si>
+    <t>${session.jury5AsTO} ${session.jury5AsTO.federation}</t>
+  </si>
+  <si>
+    <t>${session.reserveJuryAsTO} ${session.reserveJuryAsTO.federation}</t>
+  </si>
+  <si>
+    <t>${session.doctorAsTO} ${session.doctorAsTO.federation}</t>
+  </si>
+  <si>
+    <t>${session.announcerAsTO} ${session.announcerAsTO.federation}</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="ddd\ mmm\,\ d\ yyyy"/>
+  <numFmts count="1">
     <numFmt numFmtId="165" formatCode="[$-F800]dddd\,\ mmmm\ dd\,\ yyyy"/>
   </numFmts>
   <fonts count="12" x14ac:knownFonts="1">
@@ -357,7 +377,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -374,6 +394,15 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -383,9 +412,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -403,22 +429,11 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="165" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" shrinkToFit="1"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
@@ -436,10 +451,26 @@
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="165" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+      <alignment horizontal="center" vertical="top" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -790,47 +821,45 @@
     <col min="9" max="9" width="10.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" ht="28.5" x14ac:dyDescent="0.25">
-      <c r="A1" s="25" t="s">
+    <row r="1" spans="1:18" s="21" customFormat="1" ht="41.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="20" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="25"/>
-      <c r="C1" s="25"/>
-      <c r="D1" s="25"/>
-      <c r="E1" s="25"/>
-      <c r="F1" s="25"/>
-      <c r="G1" s="25"/>
-      <c r="H1" s="25"/>
-      <c r="I1" s="25"/>
-      <c r="J1" s="17"/>
-    </row>
-    <row r="2" spans="1:18" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="10"/>
-      <c r="B2" s="10"/>
-      <c r="C2" s="10"/>
-      <c r="D2" s="10"/>
-      <c r="E2" s="10"/>
-      <c r="F2" s="10"/>
-      <c r="G2" s="10"/>
-      <c r="H2" s="10"/>
-      <c r="I2" s="10"/>
+      <c r="B1" s="20"/>
+      <c r="C1" s="20"/>
+      <c r="D1" s="20"/>
+      <c r="E1" s="20"/>
+      <c r="F1" s="20"/>
+      <c r="G1" s="20"/>
+      <c r="H1" s="20"/>
+      <c r="I1" s="20"/>
+      <c r="J1" s="20"/>
+    </row>
+    <row r="2" spans="1:18" ht="23.25" x14ac:dyDescent="0.25">
+      <c r="A2" s="19" t="s">
+        <v>32</v>
+      </c>
+      <c r="B2" s="19"/>
+      <c r="C2" s="19"/>
+      <c r="D2" s="19"/>
+      <c r="E2" s="19"/>
+      <c r="F2" s="19"/>
+      <c r="G2" s="19"/>
+      <c r="H2" s="19"/>
+      <c r="I2" s="19"/>
     </row>
     <row r="3" spans="1:18" ht="23.25" x14ac:dyDescent="0.35">
-      <c r="A3" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="B3" s="15"/>
-      <c r="C3" s="12"/>
-      <c r="D3" s="24" t="s">
-        <v>9</v>
-      </c>
-      <c r="E3" s="24"/>
-      <c r="F3" s="24"/>
-      <c r="G3" s="24"/>
-      <c r="H3" s="12"/>
-      <c r="I3" s="13" t="s">
-        <v>1</v>
-      </c>
+      <c r="A3" s="18" t="s">
+        <v>33</v>
+      </c>
+      <c r="B3" s="18"/>
+      <c r="C3" s="18"/>
+      <c r="D3" s="18"/>
+      <c r="E3" s="22"/>
+      <c r="F3" s="9"/>
+      <c r="G3" s="23"/>
+      <c r="H3" s="23"/>
+      <c r="I3" s="23"/>
     </row>
     <row r="4" spans="1:18" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A4" s="2"/>
@@ -844,52 +873,54 @@
       <c r="I4" s="2"/>
     </row>
     <row r="5" spans="1:18" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="B5" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="C5" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="D5" s="9"/>
-      <c r="E5" s="5" t="s">
+      <c r="A5" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D5" s="8"/>
+      <c r="E5" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="F5" s="4"/>
+      <c r="G5" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="H5" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="F5" s="5"/>
-      <c r="G5" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="H5" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="I5" s="7"/>
+      <c r="I5" s="6"/>
+      <c r="J5" s="24"/>
     </row>
     <row r="6" spans="1:18" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="4" t="s">
+      <c r="A6" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="B6" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="B6" s="8" t="s">
+      <c r="C6" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="D6" s="7"/>
+      <c r="E6" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="C6" s="8" t="s">
-        <v>8</v>
-      </c>
-      <c r="D6" s="8"/>
-      <c r="E6" s="4" t="s">
+      <c r="F6" s="3"/>
+      <c r="G6" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="F6" s="4"/>
-      <c r="G6" s="4" t="s">
+      <c r="H6" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="H6" s="4" t="s">
+      <c r="I6" s="25" t="s">
         <v>6</v>
       </c>
-      <c r="I6" s="3" t="s">
-        <v>7</v>
-      </c>
+      <c r="J6" s="25"/>
     </row>
     <row r="7" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A7" s="1"/>
@@ -903,165 +934,172 @@
       <c r="I7" s="1"/>
     </row>
     <row r="8" spans="1:18" ht="28.5" x14ac:dyDescent="0.45">
-      <c r="B8" s="16" t="s">
-        <v>14</v>
-      </c>
-      <c r="C8" s="16"/>
-      <c r="D8" s="16"/>
-      <c r="E8" s="16"/>
-      <c r="F8" s="14"/>
-      <c r="G8" s="14"/>
-      <c r="H8" s="14"/>
-      <c r="I8" s="14"/>
+      <c r="B8" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="C8" s="11"/>
+      <c r="D8" s="11"/>
+      <c r="E8" s="11"/>
+      <c r="F8" s="10"/>
+      <c r="G8" s="10"/>
+      <c r="H8" s="10"/>
+      <c r="I8" s="10"/>
     </row>
     <row r="10" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="B10" s="18" t="s">
+      <c r="B10" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="C10" t="s">
+        <v>34</v>
+      </c>
+      <c r="F10" s="12" t="s">
         <v>24</v>
       </c>
-      <c r="C10" t="s">
+      <c r="G10" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="11" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="B11" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="C11" t="s">
+        <v>35</v>
+      </c>
+      <c r="F11" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="G11" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="12" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B12" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="C12" t="s">
+        <v>36</v>
+      </c>
+      <c r="F12" s="12" t="s">
+        <v>27</v>
+      </c>
+      <c r="G12" t="s">
+        <v>45</v>
+      </c>
+      <c r="O12" s="12"/>
+      <c r="R12" s="17"/>
+    </row>
+    <row r="13" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B13" s="12" t="s">
+        <v>18</v>
+      </c>
+      <c r="C13" t="s">
+        <v>37</v>
+      </c>
+      <c r="F13" s="12" t="s">
+        <v>28</v>
+      </c>
+      <c r="G13" t="s">
+        <v>46</v>
+      </c>
+      <c r="O13" s="12"/>
+      <c r="R13" s="17"/>
+    </row>
+    <row r="14" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="F14" s="12" t="s">
         <v>29</v>
       </c>
-      <c r="F10" s="18" t="s">
+      <c r="G14" t="s">
+        <v>47</v>
+      </c>
+      <c r="N14" s="12"/>
+      <c r="O14" s="12"/>
+      <c r="Q14" s="17"/>
+      <c r="R14" s="17"/>
+    </row>
+    <row r="15" spans="1:18" ht="24.75" x14ac:dyDescent="0.25">
+      <c r="B15" s="15" t="s">
         <v>19</v>
       </c>
-      <c r="G10" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="11" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="B11" s="18" t="s">
+      <c r="C15" t="s">
+        <v>38</v>
+      </c>
+      <c r="F15" s="12" t="s">
+        <v>25</v>
+      </c>
+      <c r="G15" t="s">
+        <v>48</v>
+      </c>
+      <c r="K15" s="13"/>
+      <c r="N15" s="16"/>
+      <c r="O15" s="13"/>
+    </row>
+    <row r="16" spans="1:18" ht="24.75" x14ac:dyDescent="0.25">
+      <c r="B16" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="C16" t="s">
         <v>39</v>
       </c>
-      <c r="C11" t="s">
+      <c r="K16" s="13"/>
+      <c r="N16" s="16"/>
+      <c r="O16" s="13"/>
+    </row>
+    <row r="17" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B17" s="15"/>
+      <c r="F17" s="12" t="s">
         <v>30</v>
       </c>
-      <c r="F11" s="18" t="s">
+      <c r="G17" t="s">
+        <v>49</v>
+      </c>
+      <c r="K17" s="14"/>
+      <c r="N17" s="12"/>
+      <c r="O17" s="12"/>
+    </row>
+    <row r="18" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B18" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="G11" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="12" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B12" s="18" t="s">
-        <v>39</v>
-      </c>
-      <c r="C12" t="s">
+      <c r="C18" t="s">
+        <v>40</v>
+      </c>
+      <c r="N18" s="12"/>
+      <c r="O18" s="12"/>
+    </row>
+    <row r="19" spans="2:15" ht="24.75" x14ac:dyDescent="0.25">
+      <c r="B19" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="C19" t="s">
+        <v>41</v>
+      </c>
+      <c r="F19" s="12" t="s">
         <v>31</v>
       </c>
-      <c r="F12" s="18" t="s">
-        <v>21</v>
-      </c>
-      <c r="G12" t="s">
-        <v>36</v>
-      </c>
-      <c r="O12" s="18"/>
-      <c r="R12" s="23"/>
-    </row>
-    <row r="13" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B13" s="18" t="s">
-        <v>40</v>
-      </c>
-      <c r="C13" t="s">
-        <v>41</v>
-      </c>
-      <c r="F13" s="18" t="s">
-        <v>21</v>
-      </c>
-      <c r="G13" t="s">
-        <v>37</v>
-      </c>
-      <c r="O13" s="18"/>
-      <c r="R13" s="23"/>
-    </row>
-    <row r="14" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="F14" s="18" t="s">
-        <v>21</v>
-      </c>
-      <c r="G14" t="s">
-        <v>38</v>
-      </c>
-      <c r="N14" s="18"/>
-      <c r="O14" s="18"/>
-      <c r="Q14" s="23"/>
-      <c r="R14" s="23"/>
-    </row>
-    <row r="15" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="B15" s="21" t="s">
-        <v>20</v>
-      </c>
-      <c r="C15" t="s">
-        <v>26</v>
-      </c>
-      <c r="F15" s="18" t="s">
+      <c r="G19" t="s">
+        <v>50</v>
+      </c>
+      <c r="N19" s="12"/>
+      <c r="O19" s="12"/>
+    </row>
+    <row r="20" spans="2:15" ht="24.75" x14ac:dyDescent="0.25">
+      <c r="B20" s="15" t="s">
+        <v>23</v>
+      </c>
+      <c r="C20" t="s">
         <v>42</v>
       </c>
-      <c r="G15" t="s">
-        <v>43</v>
-      </c>
-      <c r="K15" s="19"/>
-      <c r="N15" s="22"/>
-      <c r="O15" s="19"/>
-    </row>
-    <row r="16" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="B16" s="21" t="s">
-        <v>20</v>
-      </c>
-      <c r="C16" t="s">
-        <v>27</v>
-      </c>
-      <c r="K16" s="19"/>
-      <c r="N16" s="22"/>
-      <c r="O16" s="19"/>
-    </row>
-    <row r="17" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B17" s="21"/>
-      <c r="F17" s="18" t="s">
-        <v>18</v>
-      </c>
-      <c r="G17" t="s">
-        <v>25</v>
-      </c>
-      <c r="K17" s="20"/>
-      <c r="N17" s="18"/>
-      <c r="O17" s="18"/>
-    </row>
-    <row r="18" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B18" s="18" t="s">
-        <v>22</v>
-      </c>
-      <c r="C18" t="s">
-        <v>28</v>
-      </c>
-      <c r="N18" s="18"/>
-      <c r="O18" s="18"/>
-    </row>
-    <row r="19" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B19" s="21" t="s">
-        <v>23</v>
-      </c>
-      <c r="C19" t="s">
-        <v>32</v>
-      </c>
-      <c r="N19" s="18"/>
-      <c r="O19" s="18"/>
-    </row>
-    <row r="20" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B20" s="21" t="s">
-        <v>23</v>
-      </c>
-      <c r="C20" t="s">
-        <v>33</v>
-      </c>
-      <c r="K20" s="19"/>
+      <c r="K20" s="13"/>
     </row>
     <row r="21" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="K21" s="20"/>
+      <c r="K21" s="14"/>
     </row>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="D3:G3"/>
-    <mergeCell ref="A1:I1"/>
+  <mergeCells count="3">
+    <mergeCell ref="I6:J6"/>
+    <mergeCell ref="A2:I2"/>
+    <mergeCell ref="A1:J1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup scale="64" fitToHeight="0" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>

<commit_message>
2nd doctor on introduction sheets.
</commit_message>
<xml_diff>
--- a/owlcms/src/main/resources/templates/introduction/Introduction.xlsx
+++ b/owlcms/src/main/resources/templates/introduction/Introduction.xlsx
@@ -131,7 +131,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="52">
   <si>
     <t>${competition.competitionName}</t>
   </si>
@@ -284,6 +284,9 @@
   </si>
   <si>
     <t>${session.announcerAsTO} ${session.announcerAsTO.federation}</t>
+  </si>
+  <si>
+    <t>${session.doctor2AsTO} ${session.doctor2AsTO.federation}</t>
   </si>
 </sst>
 </file>
@@ -1064,6 +1067,9 @@
       <c r="C18" t="s">
         <v>40</v>
       </c>
+      <c r="G18" t="s">
+        <v>51</v>
+      </c>
       <c r="N18" s="12"/>
       <c r="O18" s="12"/>
     </row>
@@ -1092,9 +1098,13 @@
       </c>
       <c r="K20" s="13"/>
     </row>
-    <row r="21" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:15" x14ac:dyDescent="0.25" ht="24.75" customHeight="1">
       <c r="K21" s="14"/>
     </row>
+    <row r="22" spans="2:15" ht="24.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="23" spans="2:15" ht="24.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="24" spans="2:15" ht="24.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="25" spans="2:15" ht="24.75" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="I6:J6"/>

</xml_diff>